<commit_message>
feat(db): give each case its own course_id
A case is a course of treatment, and the same patient can have several
cases, so the case identifier must be independent of patient_id. Add a
course_id (ULID) column to info_record: a first visit generates a new
course_id and follow-ups inherit their parent's, replacing the implicit
"father_id root record" as the grouping key.

Includes an Alembic migration that backfills a ULID per existing
father_id group, the course list now groups and returns course_id plus
first_record_id (for navigation), and the structure specification
workbook is regenerated to stay in sync (248 fields).

Adds a test that two cases for one patient get distinct course_ids.
</commit_message>
<xml_diff>
--- a/docs/case-database-spec.xlsx
+++ b/docs/case-database-spec.xlsx
@@ -1,35 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00 总览" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 患者基本信息表" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 就诊信息记录表" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 带教老师表" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 病案文本记录表" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 诊断记录表" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 治疗记录表" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 处方药味明细表" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 中药字典表" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 中药别名表" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 证型字典表" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 方剂字典表" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 通用术语字典表" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 学习笔记表" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 导师点评表" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 笔记与病案关联表" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16 来源单据表" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17 附件表" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18 OCR作业表" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19 OCR字段置信度表" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20 审计日志表" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21 应用设置表" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="附表 枚举字典" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="00 总览" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="01 患者基本信息表" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="02 就诊信息记录表" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="03 带教老师表" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="04 病案文本记录表" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="05 诊断记录表" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="06 治疗记录表" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="07 处方药味明细表" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="08 中药字典表" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="09 中药别名表" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="10 证型字典表" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="11 方剂字典表" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="12 通用术语字典表" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="13 学习笔记表" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="14 导师点评表" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="15 笔记与病案关联表" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="16 来源单据表" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="17 附件表" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="18 OCR作业表" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="19 OCR字段置信度表" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="20 审计日志表" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="21 应用设置表" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="附表 枚举字典" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6272,7 +6272,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6353,12 +6353,12 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>patient_id</t>
+          <t>course_id</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>患者编号</t>
+          <t>病案编号</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -6368,51 +6368,51 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>FOREIGN KEY</t>
+          <t>NOT NULL DEFAULT ''</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>计算机生成，与患者基本信息同步记录</t>
+          <t>病案编号（病程系列），ULID。同一患者可有多个病案，病案标识独立于患者编号，不得复用 patient_id</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>father_id</t>
+          <t>patient_id</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>父节点病历编号</t>
+          <t>患者编号</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>INTEGER</t>
+          <t>TEXT</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>FOREIGN KEY NOT NULL</t>
+          <t>FOREIGN KEY</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>初诊病历的父节点编号等于其自身病历编号；复诊病历的父节点编号等于其初诊病历编号。取整个病程：WHERE father_id = ?</t>
+          <t>计算机生成，与患者基本信息同步记录</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>visit_no</t>
+          <t>father_id</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>第几诊</t>
+          <t>父节点病历编号</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -6422,83 +6422,83 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>NOT NULL DEFAULT 1</t>
+          <t>FOREIGN KEY NOT NULL</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>初诊为1，其后依次递增</t>
+          <t>初诊病历的父节点编号等于其自身病历编号；复诊病历的父节点编号等于其初诊病历编号。取整个病程：WHERE father_id = ?</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>visit_type</t>
+          <t>visit_no</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>就诊类型</t>
+          <t>第几诊</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>UNSIGNED TINYINT</t>
+          <t>INTEGER</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>DEFAULT 0</t>
+          <t>NOT NULL DEFAULT 1</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>0为初诊，1为复诊，2为随访；详见附表A2</t>
+          <t>初诊为1，其后依次递增</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>clinic_date</t>
+          <t>visit_type</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>就诊日期</t>
+          <t>就诊类型</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>DATE</t>
+          <t>UNSIGNED TINYINT</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>NOT NULL</t>
+          <t>DEFAULT 0</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>必填，以“%Y-%m-%d”形式记录</t>
+          <t>0为初诊，1为复诊，2为随访；详见附表A2</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>age</t>
+          <t>clinic_date</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>就诊年龄</t>
+          <t>就诊日期</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>REAL</t>
+          <t>DATE</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -6508,46 +6508,46 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>必填，年龄范围：[0, 200]</t>
+          <t>必填，以“%Y-%m-%d”形式记录</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>doctor_name</t>
+          <t>age</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>就诊医师</t>
+          <t>就诊年龄</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>TEXT</t>
+          <t>REAL</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>DEFAULT ''</t>
+          <t>NOT NULL</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>选填，记录原始姓名写法</t>
+          <t>必填，年龄范围：[0, 200]</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>mentor_id</t>
+          <t>doctor_name</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>带教老师编号</t>
+          <t>就诊医师</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -6557,24 +6557,24 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>FOREIGN KEY</t>
+          <t>DEFAULT ''</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>选填，关联 mentor；用于按老师统计用药与辨证规律</t>
+          <t>选填，记录原始姓名写法</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>department</t>
+          <t>mentor_id</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>就诊科室</t>
+          <t>带教老师编号</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -6584,24 +6584,24 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>DEFAULT ''</t>
+          <t>FOREIGN KEY</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>选填。注意：就诊科室不等于疾病所属专科</t>
+          <t>选填，关联 mentor；用于按老师统计用药与辨证规律</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>addr</t>
+          <t>department</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>就诊地点</t>
+          <t>就诊科室</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -6616,123 +6616,127 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>选填，如医院与门诊名称</t>
+          <t>选填。注意：就诊科室不等于疾病所属专科</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>solar_terms</t>
+          <t>addr</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>就诊节气</t>
+          <t>就诊地点</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>UNSIGNED TINYINT</t>
+          <t>TEXT</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>DEFAULT 0</t>
+          <t>DEFAULT ''</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>计算机由就诊日期推算，编号从0开始，详见附表A3</t>
+          <t>选填，如医院与门诊名称</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>source_document_id</t>
+          <t>solar_terms</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>来源单据编号</t>
+          <t>就诊节气</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>TEXT</t>
+          <t>UNSIGNED TINYINT</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>FOREIGN KEY</t>
+          <t>DEFAULT 0</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>选填，关联 source_document；手工录入时为空</t>
+          <t>计算机由就诊日期推算，编号从0开始，详见附表A3</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>is_deleted</t>
+          <t>source_document_id</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>是否删除</t>
+          <t>来源单据编号</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>BOOLEAN</t>
+          <t>TEXT</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>DEFAULT 0</t>
+          <t>FOREIGN KEY</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>软删除标记，0为正常，1为已删除</t>
+          <t>选填，关联 source_document；手工录入时为空</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>is_deleted</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>创建时间</t>
+          <t>是否删除</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>TIMESTAMP</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr"/>
+          <t>BOOLEAN</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录创建时间</t>
+          <t>软删除标记，0为正常，1为已删除</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>修改时间</t>
+          <t>创建时间</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -6742,6 +6746,29 @@
       </c>
       <c r="D19" s="4" t="inlineStr"/>
       <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录创建时间</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>修改时间</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr"/>
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录修改时间</t>
         </is>

</xml_diff>

<commit_message>
feat(db): add western_medicine field and first-visit narrative
Treatment gains a dedicated western_medicine column so western meds are
recorded separately from other_treatment (which now holds only Chinese
patent medicine, acupuncture and external therapy). Includes a migration
and the regenerated spec workbook.

The record detail now also returns first_narrative (the course's first
visit), so past history, personal history and allergies -- which are
recorded once at the first visit -- can be shown on follow-up visits. The
Word report shows western meds per visit and only repeats the first-visit
history fields on the first visit.

Adds a test covering both the western medicine round-trip and the
first-narrative fallback.
</commit_message>
<xml_diff>
--- a/docs/case-database-spec.xlsx
+++ b/docs/case-database-spec.xlsx
@@ -1,35 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="00 总览" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="01 患者基本信息表" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="02 就诊信息记录表" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="03 带教老师表" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="04 病案文本记录表" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="05 诊断记录表" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="06 治疗记录表" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="07 处方药味明细表" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="08 中药字典表" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="09 中药别名表" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="10 证型字典表" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="11 方剂字典表" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="12 通用术语字典表" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="13 学习笔记表" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="14 导师点评表" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="15 笔记与病案关联表" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="16 来源单据表" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="17 附件表" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="18 OCR作业表" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="19 OCR字段置信度表" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="20 审计日志表" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="21 应用设置表" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="附表 枚举字典" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00 总览" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 患者基本信息表" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 就诊信息记录表" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 带教老师表" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 病案文本记录表" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 诊断记录表" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 治疗记录表" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 处方药味明细表" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 中药字典表" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 中药别名表" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 证型字典表" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 方剂字典表" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 通用术语字典表" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 学习笔记表" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 导师点评表" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 笔记与病案关联表" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16 来源单据表" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17 附件表" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18 OCR作业表" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19 OCR字段置信度表" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20 审计日志表" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21 应用设置表" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="附表 枚举字典" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -8043,7 +8043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -8340,12 +8340,12 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>other_treatment</t>
+          <t>western_medicine</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>其他治疗</t>
+          <t>西药</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -8360,19 +8360,19 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>选填，自由文本。中成药、西医治疗、针灸外治等一并记于此栏</t>
+          <t>选填，自由文本，如“甲钴胺 0.5mg tid”；西药单列，不与中药混</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>raw_ocr_text</t>
+          <t>other_treatment</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>OCR 原文</t>
+          <t>其他治疗</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -8387,42 +8387,46 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>处方原文，只写不改，用于溯源</t>
+          <t>选填，自由文本。中成药、针灸外治等一并记于此栏</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>raw_ocr_text</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>创建时间</t>
+          <t>OCR 原文</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>TIMESTAMP</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr"/>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录创建时间</t>
+          <t>处方原文，只写不改，用于溯源</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>修改时间</t>
+          <t>创建时间</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -8432,6 +8436,29 @@
       </c>
       <c r="D16" s="4" t="inlineStr"/>
       <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录创建时间</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>修改时间</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr"/>
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录修改时间</t>
         </is>

</xml_diff>

<commit_message>
feat(api): add interface templates for fixed HIS layouts
Add dict_template (name, doc_type, field_anchors, table_columns) so a
user can codify the text structure and table columns of a fixed HIS
screen from a few samples. Provide CRUD endpoints, inject the template
into lane-B structuring prompts, and add a key-independent
POST /api/ocr/jobs/{id}/extract that pulls field values from lane-A text
using the anchors ("label: value" pattern) as a manual-review prefill.
</commit_message>
<xml_diff>
--- a/docs/case-database-spec.xlsx
+++ b/docs/case-database-spec.xlsx
@@ -20,16 +20,17 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 证型字典表" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 方剂字典表" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 通用术语字典表" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 学习笔记表" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 导师点评表" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 笔记与病案关联表" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16 来源单据表" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17 附件表" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18 OCR作业表" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19 OCR字段置信度表" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20 审计日志表" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21 应用设置表" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="附表 枚举字典" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 界面模板表" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 学习笔记表" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 导师点评表" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 笔记与病案关联表" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16 来源单据表" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17 附件表" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18 OCR作业表" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19 OCR字段置信度表" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20 审计日志表" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21 应用设置表" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="附表 枚举字典" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -515,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -872,22 +873,22 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>五、跟师学习</t>
+          <t>四、字典</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>learning_note</t>
+          <t>dict_template</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>学习笔记表</t>
+          <t>界面模板表</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>以 note_type 区分跟诊日志与学习心得，避免为相似结构建多张表。</t>
+          <t>固化特定 HIS 界面的文字结构与表格列，供 OCR 结构化提示与本地“按模板提取”使用，以提升固定界面的识别准确度。</t>
         </is>
       </c>
     </row>
@@ -902,17 +903,17 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>mentor_comment</t>
+          <t>learning_note</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>导师点评表</t>
+          <t>学习笔记表</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>师承关系中的权威内容。is_ai_generated 字段确保 AI 生成内容绝不被误认为真实导师点评，界面须视觉区分。</t>
+          <t>以 note_type 区分跟诊日志与学习心得，避免为相似结构建多张表。</t>
         </is>
       </c>
     </row>
@@ -927,17 +928,17 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>note_record_link</t>
+          <t>mentor_comment</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>笔记与病案关联表</t>
+          <t>导师点评表</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>学习心得与病案的双向引用，支持“从心得跳病案”与反向追溯。</t>
+          <t>师承关系中的权威内容。is_ai_generated 字段确保 AI 生成内容绝不被误认为真实导师点评，界面须视觉区分。</t>
         </is>
       </c>
     </row>
@@ -947,22 +948,22 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>六、来源与溯源</t>
+          <t>五、跟师学习</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>source_document</t>
+          <t>note_record_link</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>来源单据表</t>
+          <t>笔记与病案关联表</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>真实样本显示同一病程的数据可能来自手写教学表单、HIS 打印件或 HIS 界面截图，来源不同则解析策略与可信度不同。</t>
+          <t>学习心得与病案的双向引用，支持“从心得跳病案”与反向追溯。</t>
         </is>
       </c>
     </row>
@@ -977,17 +978,17 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>attachment</t>
+          <t>source_document</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>附件表</t>
+          <t>来源单据表</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>文件本体存于 data/attachments/，库中仅存路径与哈希。sha256 用于去重与完整性校验。</t>
+          <t>真实样本显示同一病程的数据可能来自手写教学表单、HIS 打印件或 HIS 界面截图，来源不同则解析策略与可信度不同。</t>
         </is>
       </c>
     </row>
@@ -1002,17 +1003,17 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>ocr_job</t>
+          <t>attachment</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>OCR作业表</t>
+          <t>附件表</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>一次识别的完整留痕：双通道结果、提示词版本、成本与耗时。提示词固定前缀须字节级稳定以命中 DeepSeek 上下文缓存。</t>
+          <t>文件本体存于 data/attachments/，库中仅存路径与哈希。sha256 用于去重与完整性校验。</t>
         </is>
       </c>
     </row>
@@ -1027,17 +1028,17 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>ocr_field_confidence</t>
+          <t>ocr_job</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>OCR字段置信度表</t>
+          <t>OCR作业表</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>驱动校对界面高亮，同时是 OCR 评测的数据来源。真实样本显示印刷体置信度0.5~1.0、手写体约0.3，可据此路由。</t>
+          <t>一次识别的完整留痕：双通道结果、提示词版本、成本与耗时。提示词固定前缀须字节级稳定以命中 DeepSeek 上下文缓存。</t>
         </is>
       </c>
     </row>
@@ -1047,22 +1048,22 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>七、系统</t>
+          <t>六、来源与溯源</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>audit_log</t>
+          <t>ocr_field_confidence</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>审计日志表</t>
+          <t>OCR字段置信度表</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>字段级修改留痕。学习记录的可信性依赖不可抵赖的修改历史。</t>
+          <t>驱动校对界面高亮，同时是 OCR 评测的数据来源。真实样本显示印刷体置信度0.5~1.0、手写体约0.3，可据此路由。</t>
         </is>
       </c>
     </row>
@@ -1077,15 +1078,40 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
+          <t>audit_log</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>审计日志表</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>字段级修改留痕。学习记录的可信性依赖不可抵赖的修改历史。</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>七、系统</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
           <t>app_setting</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>应用设置表</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>仅存非敏感偏好。API Key 等敏感项存于 .env，不入库、不入 Git。</t>
         </is>
@@ -2357,6 +2383,257 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>界面模板表（dict_template）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>固化特定 HIS 界面的文字结构与表格列，供 OCR 结构化提示与本地“按模板提取”使用，以提升固定界面的识别准确度。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>字段名称</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>中文释义</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>数据类型（SQLite）</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>键描述</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>数据说明与数据约束</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>template_id</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>模板编号</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>PRIMARY KEY</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>计算机生成：以ULID方式生成唯一编号</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>模板名</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>必填，如“HIS 病历界面”“HIS 医嘱界面”</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>doc_type</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>单据类型</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>UNSIGNED TINYINT</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>NOT NULL DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>0为病历，1为医嘱/处方，2为其他；详见附表A11</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>field_anchors</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>文字结构</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>JSON</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT '[]'</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>列表[{label, field}]，标签→字段路径，如 [{label:"主诉", field:"narrative.complaint"}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>table_columns</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>表格列</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>JSON</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT '[]'</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>列表[{header, field}]，表头→字段路径，用于医嘱/处方表格解析</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>is_active</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>是否启用</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>BOOLEAN</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 1</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>0为停用，1为启用</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>创建时间</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录创建时间</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2733,7 +3010,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3038,7 +3315,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3262,7 +3539,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3567,7 +3844,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4029,629 +4306,6 @@
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="62" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>OCR作业表（ocr_job）</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>一次识别的完整留痕：双通道结果、提示词版本、成本与耗时。提示词固定前缀须字节级稳定以命中 DeepSeek 上下文缓存。</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>字段名称</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>中文释义</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>数据类型（SQLite）</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>键描述</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>数据说明与数据约束</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>通道A结构化结果（vision_json）</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="n"/>
-      <c r="I3" s="8" t="inlineStr">
-        <is>
-          <t>Array[Object]</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>job_id</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>作业编号</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>PRIMARY KEY</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>计算机生成：以ULID方式生成唯一编号</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>text&lt;string&gt;</t>
-        </is>
-      </c>
-      <c r="H4" s="10" t="inlineStr">
-        <is>
-          <t>识别文本</t>
-        </is>
-      </c>
-      <c r="I4" s="11" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>attach_id</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>附件编号</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>FOREIGN KEY NOT NULL</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>必填，关联 attachment</t>
-        </is>
-      </c>
-      <c r="G5" s="9" t="inlineStr">
-        <is>
-          <t>confidence&lt;float&gt;</t>
-        </is>
-      </c>
-      <c r="H5" s="10" t="inlineStr">
-        <is>
-          <t>置信度</t>
-        </is>
-      </c>
-      <c r="I5" s="11" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>record_id</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>病历编号</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>INTEGER</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>FOREIGN KEY</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>选填，关联 info_record</t>
-        </is>
-      </c>
-      <c r="G6" s="9" t="inlineStr">
-        <is>
-          <t>bbox&lt;[float]&gt;</t>
-        </is>
-      </c>
-      <c r="H6" s="10" t="inlineStr">
-        <is>
-          <t>坐标框</t>
-        </is>
-      </c>
-      <c r="I6" s="11" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>状态</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>UNSIGNED TINYINT</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>NOT NULL DEFAULT 0</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>0为待处理，1为进行中，2为成功，3为失败，4为已校对，5为已废弃；详见附表A14</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>vision_engine</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>通道A引擎</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT 'ocrmac/Vision'</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>选填，本地 macOS Vision 引擎标识</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>vision_text</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>通道A文本</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT ''</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>选填，本地 OCR 纯文本结果</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>vision_json</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>通道A结构化结果</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>JSON</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT []</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>选填，Array[Object]，含 text、confidence、bbox 三键</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>vision_ms</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>通道A耗时</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>INTEGER</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT 0</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>选填，单位：毫秒</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>通道B模型</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT ''</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>选填，如 deepseek-flash</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>prompt_version</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>提示词版本</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT ''</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>选填，用于回归对比</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>structured_json</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>通道B结构化结果</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>JSON</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT {}</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>选填，经 JSON Output 约束的输出</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>degraded_mode</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>降级模式</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>UNSIGNED TINYINT</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT 0</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>0为双通道，1为仅通道A（离线降级）；详见附表A15</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>tokens_in</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>输入tokens</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>INTEGER</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT 0</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>选填，默认为0</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>tokens_cached</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>缓存命中tokens</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>INTEGER</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT 0</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>选填，缓存命中单价约为未命中的1/50</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>tokens_out</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>输出tokens</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>INTEGER</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT 0</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>选填，默认为0</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>cost_yuan</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>费用(元)</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>REAL</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT 0</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>选填，默认为0</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>duration_ms</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>总耗时</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>INTEGER</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT 0</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>选填，单位：毫秒</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>error_message</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>错误信息</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT ''</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>选填，失败时记录错误原因</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>创建时间</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>TIMESTAMP</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr"/>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录创建时间</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="G3:H3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5153,6 +4807,629 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>OCR作业表（ocr_job）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>一次识别的完整留痕：双通道结果、提示词版本、成本与耗时。提示词固定前缀须字节级稳定以命中 DeepSeek 上下文缓存。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>字段名称</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>中文释义</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>数据类型（SQLite）</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>键描述</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>数据说明与数据约束</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>通道A结构化结果（vision_json）</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="n"/>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Array[Object]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>job_id</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>作业编号</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>PRIMARY KEY</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>计算机生成：以ULID方式生成唯一编号</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>text&lt;string&gt;</t>
+        </is>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>识别文本</t>
+        </is>
+      </c>
+      <c r="I4" s="11" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>attach_id</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>附件编号</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>FOREIGN KEY NOT NULL</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>必填，关联 attachment</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>confidence&lt;float&gt;</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>置信度</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>record_id</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>病历编号</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>FOREIGN KEY</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>选填，关联 info_record</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>bbox&lt;[float]&gt;</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>坐标框</t>
+        </is>
+      </c>
+      <c r="I6" s="11" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>状态</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>UNSIGNED TINYINT</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>NOT NULL DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>0为待处理，1为进行中，2为成功，3为失败，4为已校对，5为已废弃；详见附表A14</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>vision_engine</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>通道A引擎</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 'ocrmac/Vision'</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>选填，本地 macOS Vision 引擎标识</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>vision_text</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>通道A文本</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>选填，本地 OCR 纯文本结果</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>vision_json</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>通道A结构化结果</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>JSON</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT []</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>选填，Array[Object]，含 text、confidence、bbox 三键</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>vision_ms</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>通道A耗时</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>选填，单位：毫秒</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>通道B模型</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>选填，如 deepseek-flash</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>prompt_version</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>提示词版本</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>选填，用于回归对比</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>structured_json</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>通道B结构化结果</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>JSON</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT {}</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>选填，经 JSON Output 约束的输出</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>degraded_mode</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>降级模式</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>UNSIGNED TINYINT</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>0为双通道，1为仅通道A（离线降级）；详见附表A15</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>tokens_in</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>输入tokens</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>选填，默认为0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>tokens_cached</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>缓存命中tokens</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>选填，缓存命中单价约为未命中的1/50</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>tokens_out</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>输出tokens</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>选填，默认为0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>cost_yuan</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>费用(元)</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>REAL</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>选填，默认为0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>duration_ms</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>总耗时</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>选填，单位：毫秒</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>error_message</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>错误信息</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>选填，失败时记录错误原因</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>创建时间</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr"/>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录创建时间</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="G3:H3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5479,7 +5756,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5788,7 +6065,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5931,7 +6208,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
feat(api): add mentor list, profile and CRUD
Add clinic_time, clinic_location and bio to mentor, then a mentors
router with dropdown options, a rich list (visit and note counts) and a
detail endpoint carrying profile fields plus per-mentor statistics
(top syndromes and recent records). CRUD endpoints round it out.
</commit_message>
<xml_diff>
--- a/docs/case-database-spec.xlsx
+++ b/docs/case-database-spec.xlsx
@@ -7066,7 +7066,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -7282,39 +7282,39 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>is_primary</t>
+          <t>clinic_time</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>是否主带教</t>
+          <t>出诊时间</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>BOOLEAN</t>
+          <t>TEXT</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>DEFAULT 0</t>
+          <t>DEFAULT ''</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>0为否，1为是</t>
+          <t>选填，如“周二、四上午”</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>notes</t>
+          <t>clinic_location</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>备注</t>
+          <t>出诊地点</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -7329,78 +7329,159 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>选填，默认为空字符串</t>
+          <t>选填，如“门诊楼3层303室”</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>is_deleted</t>
+          <t>bio</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>是否删除</t>
+          <t>导师简介</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>BOOLEAN</t>
+          <t>TEXT</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>DEFAULT 0</t>
+          <t>DEFAULT ''</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>软删除标记，0为正常，1为已删除</t>
+          <t>选填，导师的简要介绍</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>is_primary</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>创建时间</t>
+          <t>是否主带教</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>TIMESTAMP</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr"/>
+          <t>BOOLEAN</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录创建时间</t>
+          <t>0为否，1为是</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>选填，默认为空字符串</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>is_deleted</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>是否删除</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>BOOLEAN</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>软删除标记，0为正常，1为已删除</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>创建时间</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr"/>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录创建时间</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
           <t>updated_at</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>修改时间</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>TIMESTAMP</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr"/>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr"/>
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录修改时间</t>
         </is>

</xml_diff>

<commit_message>
feat(api): add structured lab results to the case record
Add lab_result (category, item, value, unit, reference range, abnormal
flag) so test results can be stored structured. Wire it into record
create/update/detail, OCR structuring prompts and commit, and the Word
report. Adds a round-trip test.
</commit_message>
<xml_diff>
--- a/docs/case-database-spec.xlsx
+++ b/docs/case-database-spec.xlsx
@@ -15,22 +15,23 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 诊断记录表" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 治疗记录表" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 处方药味明细表" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 中药字典表" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 中药别名表" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 证型字典表" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 方剂字典表" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 通用术语字典表" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 界面模板表" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 学习笔记表" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 导师点评表" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 笔记与病案关联表" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16 来源单据表" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17 附件表" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18 OCR作业表" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19 OCR字段置信度表" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20 审计日志表" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21 应用设置表" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="附表 枚举字典" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 检验检查结果表" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 中药字典表" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 中药别名表" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 证型字典表" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 方剂字典表" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 通用术语字典表" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 界面模板表" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 学习笔记表" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 导师点评表" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 笔记与病案关联表" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16 来源单据表" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17 附件表" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18 OCR作业表" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19 OCR字段置信度表" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20 审计日志表" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21 应用设置表" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="附表 枚举字典" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -516,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -748,22 +749,22 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>四、字典</t>
+          <t>三、诊断与治疗</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>dict_herb</t>
+          <t>lab_result</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>中药字典表</t>
+          <t>检验检查结果表</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>炮制品作为独立条目并指向基原：盐黄柏、醋莪术、炒酸枣仁各自成条，parent_herb_id 指向基原药材。</t>
+          <t>结构化存储化验/检查数据，一行一个项目；检验类记录结果值、单位、参考范围与异常方向，影像检查类结果值为描述/结论，可由 OCR 从化验单/检查报告中识别入库。</t>
         </is>
       </c>
     </row>
@@ -778,17 +779,17 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>dict_herb_alias</t>
+          <t>dict_herb</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>中药别名表</t>
+          <t>中药字典表</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>同名异物与同物异名的显式建模。除统计归一外，还承担 OCR 药名纠错：错误几乎全为形近字（黄芩→黄苓、黄柏→黄相），而正确写法多在字典内，可用编辑距离与拼音相似度自动建议。</t>
+          <t>炮制品作为独立条目并指向基原：盐黄柏、醋莪术、炒酸枣仁各自成条，parent_herb_id 指向基原药材。</t>
         </is>
       </c>
     </row>
@@ -803,17 +804,17 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>dict_syndrome</t>
+          <t>dict_herb_alias</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>证型字典表</t>
+          <t>中药别名表</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>证候标准化与频次统计的基础。</t>
+          <t>同名异物与同物异名的显式建模。除统计归一外，还承担 OCR 药名纠错：错误几乎全为形近字（黄芩→黄苓、黄柏→黄相），而正确写法多在字典内，可用编辑距离与拼音相似度自动建议。</t>
         </is>
       </c>
     </row>
@@ -828,17 +829,17 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>dict_formula</t>
+          <t>dict_syndrome</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>方剂字典表</t>
+          <t>证型字典表</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>用于识别处方所本的基础方，支持“方剂 vs 实际处方”的加减分析。</t>
+          <t>证候标准化与频次统计的基础。</t>
         </is>
       </c>
     </row>
@@ -853,17 +854,17 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>dict_term</t>
+          <t>dict_formula</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>通用术语字典表</t>
+          <t>方剂字典表</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>承载舌质、舌苔、脉象、炮制、煎服法、用法等轻量字典，并记录使用频次用于录入联想排序。</t>
+          <t>用于识别处方所本的基础方，支持“方剂 vs 实际处方”的加减分析。</t>
         </is>
       </c>
     </row>
@@ -878,17 +879,17 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>dict_template</t>
+          <t>dict_term</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>界面模板表</t>
+          <t>通用术语字典表</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>固化特定 HIS 界面的文字结构与表格列，供 OCR 结构化提示与本地“按模板提取”使用，以提升固定界面的识别准确度。</t>
+          <t>承载舌质、舌苔、脉象、炮制、煎服法、用法等轻量字典，并记录使用频次用于录入联想排序。</t>
         </is>
       </c>
     </row>
@@ -898,22 +899,22 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>五、跟师学习</t>
+          <t>四、字典</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>learning_note</t>
+          <t>dict_template</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>学习笔记表</t>
+          <t>界面模板表</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>以 note_type 区分跟诊日志与学习心得，避免为相似结构建多张表。</t>
+          <t>固化特定 HIS 界面的文字结构与表格列，供 OCR 结构化提示与本地“按模板提取”使用，以提升固定界面的识别准确度。</t>
         </is>
       </c>
     </row>
@@ -928,17 +929,17 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>mentor_comment</t>
+          <t>learning_note</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>导师点评表</t>
+          <t>学习笔记表</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>师承关系中的权威内容。is_ai_generated 字段确保 AI 生成内容绝不被误认为真实导师点评，界面须视觉区分。</t>
+          <t>以 note_type 区分跟诊日志与学习心得，避免为相似结构建多张表。</t>
         </is>
       </c>
     </row>
@@ -953,17 +954,17 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>note_record_link</t>
+          <t>mentor_comment</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>笔记与病案关联表</t>
+          <t>导师点评表</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>学习心得与病案的双向引用，支持“从心得跳病案”与反向追溯。</t>
+          <t>师承关系中的权威内容。is_ai_generated 字段确保 AI 生成内容绝不被误认为真实导师点评，界面须视觉区分。</t>
         </is>
       </c>
     </row>
@@ -973,22 +974,22 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>六、来源与溯源</t>
+          <t>五、跟师学习</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>source_document</t>
+          <t>note_record_link</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>来源单据表</t>
+          <t>笔记与病案关联表</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>真实样本显示同一病程的数据可能来自手写教学表单、HIS 打印件或 HIS 界面截图，来源不同则解析策略与可信度不同。</t>
+          <t>学习心得与病案的双向引用，支持“从心得跳病案”与反向追溯。</t>
         </is>
       </c>
     </row>
@@ -1003,17 +1004,17 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>attachment</t>
+          <t>source_document</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>附件表</t>
+          <t>来源单据表</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>文件本体存于 data/attachments/，库中仅存路径与哈希。sha256 用于去重与完整性校验。</t>
+          <t>真实样本显示同一病程的数据可能来自手写教学表单、HIS 打印件或 HIS 界面截图，来源不同则解析策略与可信度不同。</t>
         </is>
       </c>
     </row>
@@ -1028,17 +1029,17 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>ocr_job</t>
+          <t>attachment</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>OCR作业表</t>
+          <t>附件表</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>一次识别的完整留痕：双通道结果、提示词版本、成本与耗时。提示词固定前缀须字节级稳定以命中 DeepSeek 上下文缓存。</t>
+          <t>文件本体存于 data/attachments/，库中仅存路径与哈希。sha256 用于去重与完整性校验。</t>
         </is>
       </c>
     </row>
@@ -1053,17 +1054,17 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>ocr_field_confidence</t>
+          <t>ocr_job</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>OCR字段置信度表</t>
+          <t>OCR作业表</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>驱动校对界面高亮，同时是 OCR 评测的数据来源。真实样本显示印刷体置信度0.5~1.0、手写体约0.3，可据此路由。</t>
+          <t>一次识别的完整留痕：双通道结果、提示词版本、成本与耗时。提示词固定前缀须字节级稳定以命中 DeepSeek 上下文缓存。</t>
         </is>
       </c>
     </row>
@@ -1073,22 +1074,22 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>七、系统</t>
+          <t>六、来源与溯源</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>audit_log</t>
+          <t>ocr_field_confidence</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>审计日志表</t>
+          <t>OCR字段置信度表</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>字段级修改留痕。学习记录的可信性依赖不可抵赖的修改历史。</t>
+          <t>驱动校对界面高亮，同时是 OCR 评测的数据来源。真实样本显示印刷体置信度0.5~1.0、手写体约0.3，可据此路由。</t>
         </is>
       </c>
     </row>
@@ -1103,15 +1104,40 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
+          <t>audit_log</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>审计日志表</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>字段级修改留痕。学习记录的可信性依赖不可抵赖的修改历史。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>七、系统</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
           <t>app_setting</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>应用设置表</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E27" s="4" t="inlineStr">
         <is>
           <t>仅存非敏感偏好。API Key 等敏感项存于 .env，不入库、不入 Git。</t>
         </is>
@@ -1127,6 +1153,473 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>中药字典表（dict_herb）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>炮制品作为独立条目并指向基原：盐黄柏、醋莪术、炒酸枣仁各自成条，parent_herb_id 指向基原药材。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>字段名称</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>中文释义</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>数据类型（SQLite）</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>键描述</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>数据说明与数据约束</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>herb_id</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>药材编号</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>PRIMARY KEY</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>计算机生成：以ULID方式生成唯一编号</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>herb_name</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>标准药名</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>UNIQUE NOT NULL</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>必填，标准名，如“生地黄”“盐黄柏”</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>pinyin</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>拼音</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>选填，便于拼音检索，如 sheng di huang</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>parent_herb_id</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>基原药材编号</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>FOREIGN KEY</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>选填，自引用。炮制品指向其基原，如盐黄柏→黄柏；基原药材为空</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>is_processed</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>是否炮制品</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>BOOLEAN</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>0为基原药材，1为炮制品</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>processing</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>炮制方法</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>选填，炮制品的炮制方法，如盐炙、醋炙、炒、砂烫</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>类别</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>选填，如解表药、清热药、补虚药</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>nature</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>四气</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>选填，寒、热、温、凉、平</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>flavor</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>五味</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>选填，辛、甘、酸、苦、咸、淡、涩</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>meridians</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>归经</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>选填，多条以逗号分隔</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>functions</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>功效</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>选填，默认为空字符串</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>standard_code</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>标准编码</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>选填，药典或国标编码，仅作建议不强制</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>is_common</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>是否常用药</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>BOOLEAN</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 1</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>0为否，1为是；影响录入联想排序</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>is_active</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>是否启用</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>BOOLEAN</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 1</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>0为停用，1为启用</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>创建时间</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr"/>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录创建时间</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1377,7 +1870,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1709,7 +2202,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2095,7 +2588,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2377,7 +2870,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2628,7 +3121,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3010,7 +3503,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3315,7 +3808,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3539,7 +4032,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3830,473 +4323,6 @@
       </c>
       <c r="D12" s="4" t="inlineStr"/>
       <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录创建时间</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="62" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>附件表（attachment）</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>文件本体存于 data/attachments/，库中仅存路径与哈希。sha256 用于去重与完整性校验。</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>字段名称</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>中文释义</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>数据类型（SQLite）</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>键描述</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>数据说明与数据约束</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>attach_id</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>附件编号</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>PRIMARY KEY</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>计算机生成：以ULID方式生成唯一编号</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>record_id</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>病历编号</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>INTEGER</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>FOREIGN KEY</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>选填，可先上传后关联</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>doc_id</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>单据编号</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>FOREIGN KEY</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>选填，关联 source_document</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>file_path</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>文件路径</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>必填，相对 data/ 的路径</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>thumb_path</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>缩略图路径</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT ''</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>选填，默认为空字符串</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>file_type</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>文件类型</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>UNSIGNED TINYINT</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>0为图片，1为PDF；详见附表A13</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>mime_type</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>MIME类型</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT ''</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>选填，按文件实际内容判断</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>file_size</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>文件大小</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>INTEGER</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT 0</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>选填，单位：字节</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>width</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>宽度</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>INTEGER</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT 0</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>选填，单位：像素</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>height</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>高度</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>INTEGER</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT 0</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>选填，单位：像素</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>sha256</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>文件哈希</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT ''</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>选填，用于去重与完整性校验</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>page_no</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>页码</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>INTEGER</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT 1</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>选填，多页单据中的页码</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>sort_order</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>排序</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>INTEGER</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT 0</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>选填，同一病历内附件的排列顺序</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>is_deleted</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>是否删除</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>BOOLEAN</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT 0</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>软删除标记，0为正常，1为已删除</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>创建时间</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>TIMESTAMP</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr"/>
-      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录创建时间</t>
         </is>
@@ -4807,6 +4833,473 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>附件表（attachment）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>文件本体存于 data/attachments/，库中仅存路径与哈希。sha256 用于去重与完整性校验。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>字段名称</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>中文释义</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>数据类型（SQLite）</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>键描述</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>数据说明与数据约束</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>attach_id</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>附件编号</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>PRIMARY KEY</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>计算机生成：以ULID方式生成唯一编号</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>record_id</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>病历编号</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>FOREIGN KEY</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>选填，可先上传后关联</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>doc_id</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>单据编号</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>FOREIGN KEY</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>选填，关联 source_document</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>file_path</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>文件路径</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>必填，相对 data/ 的路径</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>thumb_path</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>缩略图路径</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>选填，默认为空字符串</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>file_type</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>文件类型</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>UNSIGNED TINYINT</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>0为图片，1为PDF；详见附表A13</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>mime_type</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>MIME类型</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>选填，按文件实际内容判断</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>file_size</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>文件大小</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>选填，单位：字节</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>宽度</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>选填，单位：像素</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>height</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>高度</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>选填，单位：像素</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>sha256</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>文件哈希</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>选填，用于去重与完整性校验</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>page_no</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>页码</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 1</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>选填，多页单据中的页码</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>sort_order</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>排序</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>选填，同一病历内附件的排列顺序</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>is_deleted</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>是否删除</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>BOOLEAN</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>软删除标记，0为正常，1为已删除</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>创建时间</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr"/>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录创建时间</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5424,7 +5917,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5756,7 +6249,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6065,7 +6558,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6208,13 +6701,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6532,6 +7025,23 @@
       <c r="C19" s="4" t="inlineStr">
         <is>
           <t>0=新增；1=修改；2=删除；3=恢复；4=脱敏</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>A18</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>检验检查类别（lab_result.category）</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>0=检验；1=影像检查；2=其他</t>
         </is>
       </c>
     </row>
@@ -9385,7 +9895,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -9398,14 +9908,14 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>中药字典表（dict_herb）</t>
+          <t>检验检查结果表（lab_result）</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>炮制品作为独立条目并指向基原：盐黄柏、醋莪术、炒酸枣仁各自成条，parent_herb_id 指向基原药材。</t>
+          <t>结构化存储化验/检查数据，一行一个项目；检验类记录结果值、单位、参考范围与异常方向，影像检查类结果值为描述/结论，可由 OCR 从化验单/检查报告中识别入库。</t>
         </is>
       </c>
     </row>
@@ -9439,66 +9949,66 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>herb_id</t>
+          <t>result_id</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>药材编号</t>
+          <t>结果编号</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>TEXT</t>
+          <t>INTEGER</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>PRIMARY KEY</t>
+          <t>PRIMARY KEY AUTOINCREMENT</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>计算机生成：以ULID方式生成唯一编号</t>
+          <t>计算机生成：从1开始，以1为步长增序编号</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>herb_name</t>
+          <t>record_id</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>标准药名</t>
+          <t>病历编号</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>TEXT</t>
+          <t>INTEGER</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>UNIQUE NOT NULL</t>
+          <t>FOREIGN KEY</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>必填，标准名，如“生地黄”“盐黄柏”</t>
+          <t>必填，关联 info_record</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>pinyin</t>
+          <t>patient_id</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>拼音</t>
+          <t>患者编号</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -9508,78 +10018,78 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>DEFAULT ''</t>
+          <t>FOREIGN KEY</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>选填，便于拼音检索，如 sheng di huang</t>
+          <t>计算机生成，与患者基本信息同步记录</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>parent_herb_id</t>
+          <t>category</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>基原药材编号</t>
+          <t>类别</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>TEXT</t>
+          <t>UNSIGNED TINYINT</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>FOREIGN KEY</t>
+          <t>NOT NULL DEFAULT 0</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>选填，自引用。炮制品指向其基原，如盐黄柏→黄柏；基原药材为空</t>
+          <t>0检验，1影像检查，2其他；详见附表A18</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>is_processed</t>
+          <t>item_name</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>是否炮制品</t>
+          <t>项目名称</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>BOOLEAN</t>
+          <t>TEXT</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>DEFAULT 0</t>
+          <t>NOT NULL</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>0为基原药材，1为炮制品</t>
+          <t>必填，如“白细胞计数”“胸部CT”</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>processing</t>
+          <t>result_value</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>炮制方法</t>
+          <t>结果值</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -9594,19 +10104,19 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>选填，炮制品的炮制方法，如盐炙、醋炙、炒、砂烫</t>
+          <t>检验为数值/定性结果，影像检查为描述/结论</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>类别</t>
+          <t>单位</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -9621,19 +10131,19 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>选填，如解表药、清热药、补虚药</t>
+          <t>选填，如“10^9/L”</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>nature</t>
+          <t>reference_range</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>四气</t>
+          <t>参考范围</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -9648,190 +10158,109 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>选填，寒、热、温、凉、平</t>
+          <t>选填，如“3.5-9.5”</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>flavor</t>
+          <t>abnormal_flag</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>五味</t>
+          <t>异常方向</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>TEXT</t>
+          <t>UNSIGNED TINYINT</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>DEFAULT ''</t>
+          <t>DEFAULT 0</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>选填，辛、甘、酸、苦、咸、淡、涩</t>
+          <t>0正常，1偏高，2偏低</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>meridians</t>
+          <t>needs_review</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>归经</t>
+          <t>是否待校对</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>TEXT</t>
+          <t>BOOLEAN</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>DEFAULT ''</t>
+          <t>DEFAULT 0</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>选填，多条以逗号分隔</t>
+          <t>0为正常，1为需人工复核</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>functions</t>
+          <t>confidence</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>功效</t>
+          <t>识别置信度</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>TEXT</t>
+          <t>REAL</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>DEFAULT ''</t>
+          <t>DEFAULT 1</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>选填，默认为空字符串</t>
+          <t>选填，人工录入为1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>standard_code</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>标准编码</t>
+          <t>创建时间</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT ''</t>
-        </is>
-      </c>
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr"/>
       <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>选填，药典或国标编码，仅作建议不强制</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>is_common</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>是否常用药</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>BOOLEAN</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT 1</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>0为否，1为是；影响录入联想排序</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>is_active</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>是否启用</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>BOOLEAN</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT 1</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>0为停用，1为启用</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>创建时间</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>TIMESTAMP</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr"/>
-      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录创建时间</t>
         </is>

</xml_diff>

<commit_message>
feat(api): split lab tests and exam reports into two tables
lab_result drops the category column and becomes a pure lab-test table
(item, value, unit, reference range, abnormal flag); a new exam_report
table stores exam name, findings and conclusion. Wire both through
create/update/detail, OCR structuring and commit, and the Word report.
</commit_message>
<xml_diff>
--- a/docs/case-database-spec.xlsx
+++ b/docs/case-database-spec.xlsx
@@ -15,23 +15,24 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 诊断记录表" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 治疗记录表" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 处方药味明细表" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 检验检查结果表" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 中药字典表" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 中药别名表" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 证型字典表" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 方剂字典表" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 通用术语字典表" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 界面模板表" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 学习笔记表" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 导师点评表" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 笔记与病案关联表" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16 来源单据表" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17 附件表" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18 OCR作业表" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19 OCR字段置信度表" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20 审计日志表" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21 应用设置表" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="附表 枚举字典" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 检验结果表" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 检查报告表" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 中药字典表" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 中药别名表" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 证型字典表" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 方剂字典表" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 通用术语字典表" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 界面模板表" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 学习笔记表" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 导师点评表" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 笔记与病案关联表" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16 来源单据表" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17 附件表" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18 OCR作业表" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19 OCR字段置信度表" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20 审计日志表" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21 应用设置表" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="附表 枚举字典" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -517,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -759,12 +760,12 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>检验检查结果表</t>
+          <t>检验结果表</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>结构化存储化验/检查数据，一行一个项目；检验类记录结果值、单位、参考范围与异常方向，影像检查类结果值为描述/结论，可由 OCR 从化验单/检查报告中识别入库。</t>
+          <t>结构化存储化验数据，一行一个检验项目：结果值、单位、参考范围与异常方向。可由 OCR 从化验单中识别入库。</t>
         </is>
       </c>
     </row>
@@ -774,22 +775,22 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>四、字典</t>
+          <t>三、诊断与治疗</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>dict_herb</t>
+          <t>exam_report</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>中药字典表</t>
+          <t>检查报告表</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>炮制品作为独立条目并指向基原：盐黄柏、醋莪术、炒酸枣仁各自成条，parent_herb_id 指向基原药材。</t>
+          <t>结构化存储影像/超声/内镜等检查，一行一项：检查名称、检查所见与结论。可由 OCR 从检查报告中识别入库。</t>
         </is>
       </c>
     </row>
@@ -804,17 +805,17 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>dict_herb_alias</t>
+          <t>dict_herb</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>中药别名表</t>
+          <t>中药字典表</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>同名异物与同物异名的显式建模。除统计归一外，还承担 OCR 药名纠错：错误几乎全为形近字（黄芩→黄苓、黄柏→黄相），而正确写法多在字典内，可用编辑距离与拼音相似度自动建议。</t>
+          <t>炮制品作为独立条目并指向基原：盐黄柏、醋莪术、炒酸枣仁各自成条，parent_herb_id 指向基原药材。</t>
         </is>
       </c>
     </row>
@@ -829,17 +830,17 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>dict_syndrome</t>
+          <t>dict_herb_alias</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>证型字典表</t>
+          <t>中药别名表</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>证候标准化与频次统计的基础。</t>
+          <t>同名异物与同物异名的显式建模。除统计归一外，还承担 OCR 药名纠错：错误几乎全为形近字（黄芩→黄苓、黄柏→黄相），而正确写法多在字典内，可用编辑距离与拼音相似度自动建议。</t>
         </is>
       </c>
     </row>
@@ -854,17 +855,17 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>dict_formula</t>
+          <t>dict_syndrome</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>方剂字典表</t>
+          <t>证型字典表</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>用于识别处方所本的基础方，支持“方剂 vs 实际处方”的加减分析。</t>
+          <t>证候标准化与频次统计的基础。</t>
         </is>
       </c>
     </row>
@@ -879,17 +880,17 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>dict_term</t>
+          <t>dict_formula</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>通用术语字典表</t>
+          <t>方剂字典表</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>承载舌质、舌苔、脉象、炮制、煎服法、用法等轻量字典，并记录使用频次用于录入联想排序。</t>
+          <t>用于识别处方所本的基础方，支持“方剂 vs 实际处方”的加减分析。</t>
         </is>
       </c>
     </row>
@@ -904,17 +905,17 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>dict_template</t>
+          <t>dict_term</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>界面模板表</t>
+          <t>通用术语字典表</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>固化特定 HIS 界面的文字结构与表格列，供 OCR 结构化提示与本地“按模板提取”使用，以提升固定界面的识别准确度。</t>
+          <t>承载舌质、舌苔、脉象、炮制、煎服法、用法等轻量字典，并记录使用频次用于录入联想排序。</t>
         </is>
       </c>
     </row>
@@ -924,22 +925,22 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>五、跟师学习</t>
+          <t>四、字典</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>learning_note</t>
+          <t>dict_template</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>学习笔记表</t>
+          <t>界面模板表</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>以 note_type 区分跟诊日志与学习心得，避免为相似结构建多张表。</t>
+          <t>固化特定 HIS 界面的文字结构与表格列，供 OCR 结构化提示与本地“按模板提取”使用，以提升固定界面的识别准确度。</t>
         </is>
       </c>
     </row>
@@ -954,17 +955,17 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>mentor_comment</t>
+          <t>learning_note</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>导师点评表</t>
+          <t>学习笔记表</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>师承关系中的权威内容。is_ai_generated 字段确保 AI 生成内容绝不被误认为真实导师点评，界面须视觉区分。</t>
+          <t>以 note_type 区分跟诊日志与学习心得，避免为相似结构建多张表。</t>
         </is>
       </c>
     </row>
@@ -979,17 +980,17 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>note_record_link</t>
+          <t>mentor_comment</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>笔记与病案关联表</t>
+          <t>导师点评表</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>学习心得与病案的双向引用，支持“从心得跳病案”与反向追溯。</t>
+          <t>师承关系中的权威内容。is_ai_generated 字段确保 AI 生成内容绝不被误认为真实导师点评，界面须视觉区分。</t>
         </is>
       </c>
     </row>
@@ -999,22 +1000,22 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>六、来源与溯源</t>
+          <t>五、跟师学习</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>source_document</t>
+          <t>note_record_link</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>来源单据表</t>
+          <t>笔记与病案关联表</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>真实样本显示同一病程的数据可能来自手写教学表单、HIS 打印件或 HIS 界面截图，来源不同则解析策略与可信度不同。</t>
+          <t>学习心得与病案的双向引用，支持“从心得跳病案”与反向追溯。</t>
         </is>
       </c>
     </row>
@@ -1029,17 +1030,17 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>attachment</t>
+          <t>source_document</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>附件表</t>
+          <t>来源单据表</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>文件本体存于 data/attachments/，库中仅存路径与哈希。sha256 用于去重与完整性校验。</t>
+          <t>真实样本显示同一病程的数据可能来自手写教学表单、HIS 打印件或 HIS 界面截图，来源不同则解析策略与可信度不同。</t>
         </is>
       </c>
     </row>
@@ -1054,17 +1055,17 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>ocr_job</t>
+          <t>attachment</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>OCR作业表</t>
+          <t>附件表</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>一次识别的完整留痕：双通道结果、提示词版本、成本与耗时。提示词固定前缀须字节级稳定以命中 DeepSeek 上下文缓存。</t>
+          <t>文件本体存于 data/attachments/，库中仅存路径与哈希。sha256 用于去重与完整性校验。</t>
         </is>
       </c>
     </row>
@@ -1079,17 +1080,17 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>ocr_field_confidence</t>
+          <t>ocr_job</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>OCR字段置信度表</t>
+          <t>OCR作业表</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>驱动校对界面高亮，同时是 OCR 评测的数据来源。真实样本显示印刷体置信度0.5~1.0、手写体约0.3，可据此路由。</t>
+          <t>一次识别的完整留痕：双通道结果、提示词版本、成本与耗时。提示词固定前缀须字节级稳定以命中 DeepSeek 上下文缓存。</t>
         </is>
       </c>
     </row>
@@ -1099,22 +1100,22 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>七、系统</t>
+          <t>六、来源与溯源</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>audit_log</t>
+          <t>ocr_field_confidence</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>审计日志表</t>
+          <t>OCR字段置信度表</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>字段级修改留痕。学习记录的可信性依赖不可抵赖的修改历史。</t>
+          <t>驱动校对界面高亮，同时是 OCR 评测的数据来源。真实样本显示印刷体置信度0.5~1.0、手写体约0.3，可据此路由。</t>
         </is>
       </c>
     </row>
@@ -1129,15 +1130,40 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
+          <t>audit_log</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>审计日志表</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>字段级修改留痕。学习记录的可信性依赖不可抵赖的修改历史。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>七、系统</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
           <t>app_setting</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>应用设置表</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="E28" s="4" t="inlineStr">
         <is>
           <t>仅存非敏感偏好。API Key 等敏感项存于 .env，不入库、不入 Git。</t>
         </is>
@@ -1153,6 +1179,311 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>检查报告表（exam_report）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>结构化存储影像/超声/内镜等检查，一行一项：检查名称、检查所见与结论。可由 OCR 从检查报告中识别入库。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>字段名称</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>中文释义</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>数据类型（SQLite）</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>键描述</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>数据说明与数据约束</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>exam_id</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>检查编号</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>PRIMARY KEY AUTOINCREMENT</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>计算机生成：从1开始，以1为步长增序编号</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>record_id</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>病历编号</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>FOREIGN KEY</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>必填，关联 info_record</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>patient_id</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>患者编号</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>FOREIGN KEY</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>计算机生成，与患者基本信息同步记录</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>item_name</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>检查名称</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>必填，如“胸部CT平扫”“腹部超声”</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>finding</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>检查所见</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>选填，如“右肺上叶小结节，直径约4mm”</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>conclusion</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>结论</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>选填，诊断意见，如“右肺小结节，建议随访”</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>needs_review</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>是否待校对</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>BOOLEAN</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>0为正常，1为需人工复核</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>confidence</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>识别置信度</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>REAL</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 1</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>选填，人工录入为1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>创建时间</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr"/>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录创建时间</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1619,7 +1950,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1870,7 +2201,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2202,7 +2533,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2588,7 +2919,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2870,7 +3201,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3121,7 +3452,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3503,7 +3834,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3808,7 +4139,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4018,311 +4349,6 @@
       </c>
       <c r="D9" s="4" t="inlineStr"/>
       <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录创建时间</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="62" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>来源单据表（source_document）</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>真实样本显示同一病程的数据可能来自手写教学表单、HIS 打印件或 HIS 界面截图，来源不同则解析策略与可信度不同。</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>字段名称</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>中文释义</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>数据类型（SQLite）</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>键描述</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>数据说明与数据约束</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>doc_id</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>单据编号</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>PRIMARY KEY</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>计算机生成：以ULID方式生成唯一编号</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>doc_type</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>单据类型</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>UNSIGNED TINYINT</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>0为手写教学表单，1为HIS门诊病历，2为HIS医嘱截图，3为检验报告，4为其他；详见附表A11</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>template_name</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>表单模板名</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT ''</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>选填，如“跟师学习临床医案”“门诊病历”</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>hospital</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>机构名称</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT ''</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>选填，如医院名称</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>page_count</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>页数</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>INTEGER</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT 1</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>选填，默认为1</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>ocr_strategy</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>解析策略</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>UNSIGNED TINYINT</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT 0</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>0为手写模式，1为印刷表格模式，2为混合模式；详见附表A12</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>file_name_origin</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>原始文件名</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT ''</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>选填。真实样本的文件名形如“日期-患者-主病”，可辅助推断元数据</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>notes</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>备注</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT ''</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>选填，默认为空字符串</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>创建时间</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>TIMESTAMP</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr"/>
-      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录创建时间</t>
         </is>
@@ -4833,6 +4859,311 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>来源单据表（source_document）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>真实样本显示同一病程的数据可能来自手写教学表单、HIS 打印件或 HIS 界面截图，来源不同则解析策略与可信度不同。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>字段名称</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>中文释义</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>数据类型（SQLite）</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>键描述</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>数据说明与数据约束</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>doc_id</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>单据编号</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>PRIMARY KEY</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>计算机生成：以ULID方式生成唯一编号</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>doc_type</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>单据类型</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>UNSIGNED TINYINT</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>0为手写教学表单，1为HIS门诊病历，2为HIS医嘱截图，3为检验报告，4为其他；详见附表A11</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>template_name</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>表单模板名</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>选填，如“跟师学习临床医案”“门诊病历”</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>机构名称</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>选填，如医院名称</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>page_count</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>页数</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 1</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>选填，默认为1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>ocr_strategy</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>解析策略</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>UNSIGNED TINYINT</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>0为手写模式，1为印刷表格模式，2为混合模式；详见附表A12</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>file_name_origin</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>原始文件名</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>选填。真实样本的文件名形如“日期-患者-主病”，可辅助推断元数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>选填，默认为空字符串</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>创建时间</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr"/>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录创建时间</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5294,7 +5625,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5917,7 +6248,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6249,7 +6580,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6558,7 +6889,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6701,13 +7032,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7025,23 +7356,6 @@
       <c r="C19" s="4" t="inlineStr">
         <is>
           <t>0=新增；1=修改；2=删除；3=恢复；4=脱敏</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>A18</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>检验检查类别（lab_result.category）</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>0=检验；1=影像检查；2=其他</t>
         </is>
       </c>
     </row>
@@ -9895,7 +10209,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -9908,14 +10222,14 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>检验检查结果表（lab_result）</t>
+          <t>检验结果表（lab_result）</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>结构化存储化验/检查数据，一行一个项目；检验类记录结果值、单位、参考范围与异常方向，影像检查类结果值为描述/结论，可由 OCR 从化验单/检查报告中识别入库。</t>
+          <t>结构化存储化验数据，一行一个检验项目：结果值、单位、参考范围与异常方向。可由 OCR 从化验单中识别入库。</t>
         </is>
       </c>
     </row>
@@ -10030,39 +10344,39 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>item_name</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>类别</t>
+          <t>项目名称</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>UNSIGNED TINYINT</t>
+          <t>TEXT</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>NOT NULL DEFAULT 0</t>
+          <t>NOT NULL</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>0检验，1影像检查，2其他；详见附表A18</t>
+          <t>必填，如“白细胞计数”“血红蛋白”</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>item_name</t>
+          <t>result_value</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>项目名称</t>
+          <t>结果值</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -10072,24 +10386,24 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>NOT NULL</t>
+          <t>DEFAULT ''</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>必填，如“白细胞计数”“胸部CT”</t>
+          <t>数值或定性结果，如“12.5”“阴性”</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>result_value</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>结果值</t>
+          <t>单位</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -10104,19 +10418,19 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>检验为数值/定性结果，影像检查为描述/结论</t>
+          <t>选填，如“10^9/L”</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>reference_range</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>单位</t>
+          <t>参考范围</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -10131,51 +10445,51 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>选填，如“10^9/L”</t>
+          <t>选填，如“3.5-9.5”</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>reference_range</t>
+          <t>abnormal_flag</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>参考范围</t>
+          <t>异常方向</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>TEXT</t>
+          <t>UNSIGNED TINYINT</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>DEFAULT ''</t>
+          <t>DEFAULT 0</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>选填，如“3.5-9.5”</t>
+          <t>0正常，1偏高，2偏低</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>abnormal_flag</t>
+          <t>needs_review</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>异常方向</t>
+          <t>是否待校对</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>UNSIGNED TINYINT</t>
+          <t>BOOLEAN</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -10185,82 +10499,55 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>0正常，1偏高，2偏低</t>
+          <t>0为正常，1为需人工复核</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>confidence</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>是否待校对</t>
+          <t>识别置信度</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>BOOLEAN</t>
+          <t>REAL</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>DEFAULT 0</t>
+          <t>DEFAULT 1</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>0为正常，1为需人工复核</t>
+          <t>选填，人工录入为1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>confidence</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>识别置信度</t>
+          <t>创建时间</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>REAL</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT 1</t>
-        </is>
-      </c>
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr"/>
       <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>选填，人工录入为1</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>创建时间</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>TIMESTAMP</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr"/>
-      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录创建时间</t>
         </is>

</xml_diff>

<commit_message>
feat(api): auto-collect new dictionary terms when saving a case
On case create and update, collect herbs, syndromes and tongue/pulse
terms that fail dictionary resolution into the dictionary with an
is_auto flag (new herbs default to non-common so they don't crowd the
autocomplete). List endpoints expose the flag. Adds a round-trip test.
</commit_message>
<xml_diff>
--- a/docs/case-database-spec.xlsx
+++ b/docs/case-database-spec.xlsx
@@ -1489,7 +1489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1921,21 +1921,48 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
+          <t>is_auto</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>是否自动收集</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>BOOLEAN</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>0为手动维护，1为录入病案时自动登记的新药名</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>创建时间</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>TIMESTAMP</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr"/>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr"/>
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录创建时间</t>
         </is>
@@ -2207,7 +2234,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2504,21 +2531,48 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
+          <t>is_auto</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>是否自动收集</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>BOOLEAN</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>0为手动维护，1为录入病案时自动登记的新证型</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>创建时间</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>TIMESTAMP</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr"/>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr"/>
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录创建时间</t>
         </is>
@@ -2925,7 +2979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3189,6 +3243,33 @@
       <c r="E11" s="4" t="inlineStr">
         <is>
           <t>0为停用，1为启用</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>is_auto</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>是否自动收集</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>BOOLEAN</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>0为手动维护，1为录入病案时自动登记的新术语</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(api): add a test name to group lab results
lab_result gains test_name (e.g. 血常规/肝功能) so indicators on one
panel can be grouped. Wire it through create/update/review/detail, the
OCR structuring prompt and the Word report, which now emits a 检验名称
column when any result has one.
</commit_message>
<xml_diff>
--- a/docs/case-database-spec.xlsx
+++ b/docs/case-database-spec.xlsx
@@ -10290,7 +10290,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -10425,12 +10425,12 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>item_name</t>
+          <t>test_name</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>项目名称</t>
+          <t>检验名称</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -10440,24 +10440,24 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>NOT NULL</t>
+          <t>DEFAULT ''</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>必填，如“白细胞计数”“血红蛋白”</t>
+          <t>选填，如“血常规”“肝功能”；用于把同一张化验单的项目分组</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>result_value</t>
+          <t>item_name</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>结果值</t>
+          <t>项目名称</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -10467,24 +10467,24 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>DEFAULT ''</t>
+          <t>NOT NULL</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>数值或定性结果，如“12.5”“阴性”</t>
+          <t>必填，如“白细胞计数”“血红蛋白”</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>result_value</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>单位</t>
+          <t>结果值</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -10499,19 +10499,19 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>选填，如“10^9/L”</t>
+          <t>数值或定性结果，如“12.5”“阴性”</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>reference_range</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>参考范围</t>
+          <t>单位</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -10526,51 +10526,51 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>选填，如“3.5-9.5”</t>
+          <t>选填，如“10^9/L”</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>abnormal_flag</t>
+          <t>reference_range</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>异常方向</t>
+          <t>参考范围</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>UNSIGNED TINYINT</t>
+          <t>TEXT</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>DEFAULT 0</t>
+          <t>DEFAULT ''</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>0正常，1偏高，2偏低</t>
+          <t>选填，如“3.5-9.5”</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>abnormal_flag</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>是否待校对</t>
+          <t>异常方向</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>BOOLEAN</t>
+          <t>UNSIGNED TINYINT</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -10580,55 +10580,82 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>0为正常，1为需人工复核</t>
+          <t>0正常，1偏高，2偏低</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>confidence</t>
+          <t>needs_review</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>识别置信度</t>
+          <t>是否待校对</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>REAL</t>
+          <t>BOOLEAN</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>DEFAULT 1</t>
+          <t>DEFAULT 0</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>选填，人工录入为1</t>
+          <t>0为正常，1为需人工复核</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
+          <t>confidence</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>识别置信度</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>REAL</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 1</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>选填，人工录入为1</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>创建时间</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>TIMESTAMP</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr"/>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr"/>
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录创建时间</t>
         </is>

</xml_diff>

<commit_message>
feat(api): structure the western medicine prescription
Add western_medicine_item (drug, dose, route, frequency, days) and wire
it through create/update/review/detail, the OCR structuring prompt and
commit, the AI case context, and the Word report (now a 西药处方 table).
Seed term types 12 (route) and 13 (frequency). Adds a round-trip test.
</commit_message>
<xml_diff>
--- a/docs/case-database-spec.xlsx
+++ b/docs/case-database-spec.xlsx
@@ -17,22 +17,23 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 处方药味明细表" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 检验结果表" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 检查报告表" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 中药字典表" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 中药别名表" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 证型字典表" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 方剂字典表" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 通用术语字典表" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 界面模板表" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 学习笔记表" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 导师点评表" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 笔记与病案关联表" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16 来源单据表" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17 附件表" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18 OCR作业表" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19 OCR字段置信度表" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20 审计日志表" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21 应用设置表" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="附表 枚举字典" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 西药明细表" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 中药字典表" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 中药别名表" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 证型字典表" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 方剂字典表" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 通用术语字典表" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 界面模板表" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 学习笔记表" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 导师点评表" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 笔记与病案关联表" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16 来源单据表" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17 附件表" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18 OCR作业表" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19 OCR字段置信度表" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20 审计日志表" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21 应用设置表" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="附表 枚举字典" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -518,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -800,22 +801,22 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>四、字典</t>
+          <t>三、诊断与治疗</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>dict_herb</t>
+          <t>western_medicine_item</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>中药字典表</t>
+          <t>西药明细表</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>炮制品作为独立条目并指向基原：盐黄柏、醋莪术、炒酸枣仁各自成条，parent_herb_id 指向基原药材。</t>
+          <t>结构化存储西药处方，一行一味：药名、剂量、给药途径、给药频次与天数。可由 OCR 从医嘱单中识别入库。</t>
         </is>
       </c>
     </row>
@@ -830,17 +831,17 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>dict_herb_alias</t>
+          <t>dict_herb</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>中药别名表</t>
+          <t>中药字典表</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>同名异物与同物异名的显式建模。除统计归一外，还承担 OCR 药名纠错：错误几乎全为形近字（黄芩→黄苓、黄柏→黄相），而正确写法多在字典内，可用编辑距离与拼音相似度自动建议。</t>
+          <t>炮制品作为独立条目并指向基原：盐黄柏、醋莪术、炒酸枣仁各自成条，parent_herb_id 指向基原药材。</t>
         </is>
       </c>
     </row>
@@ -855,17 +856,17 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>dict_syndrome</t>
+          <t>dict_herb_alias</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>证型字典表</t>
+          <t>中药别名表</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>证候标准化与频次统计的基础。</t>
+          <t>同名异物与同物异名的显式建模。除统计归一外，还承担 OCR 药名纠错：错误几乎全为形近字（黄芩→黄苓、黄柏→黄相），而正确写法多在字典内，可用编辑距离与拼音相似度自动建议。</t>
         </is>
       </c>
     </row>
@@ -880,17 +881,17 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>dict_formula</t>
+          <t>dict_syndrome</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>方剂字典表</t>
+          <t>证型字典表</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>用于识别处方所本的基础方，支持“方剂 vs 实际处方”的加减分析。</t>
+          <t>证候标准化与频次统计的基础。</t>
         </is>
       </c>
     </row>
@@ -905,17 +906,17 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>dict_term</t>
+          <t>dict_formula</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>通用术语字典表</t>
+          <t>方剂字典表</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>承载舌质、舌苔、脉象、炮制、煎服法、用法等轻量字典，并记录使用频次用于录入联想排序。</t>
+          <t>用于识别处方所本的基础方，支持“方剂 vs 实际处方”的加减分析。</t>
         </is>
       </c>
     </row>
@@ -930,17 +931,17 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>dict_template</t>
+          <t>dict_term</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>界面模板表</t>
+          <t>通用术语字典表</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>固化特定 HIS 界面的文字结构与表格列，供 OCR 结构化提示与本地“按模板提取”使用，以提升固定界面的识别准确度。</t>
+          <t>承载舌质、舌苔、脉象、炮制、煎服法、用法等轻量字典，并记录使用频次用于录入联想排序。</t>
         </is>
       </c>
     </row>
@@ -950,22 +951,22 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>五、跟师学习</t>
+          <t>四、字典</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>learning_note</t>
+          <t>dict_template</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>学习笔记表</t>
+          <t>界面模板表</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>以 note_type 区分跟诊日志与学习心得，避免为相似结构建多张表。</t>
+          <t>固化特定 HIS 界面的文字结构与表格列，供 OCR 结构化提示与本地“按模板提取”使用，以提升固定界面的识别准确度。</t>
         </is>
       </c>
     </row>
@@ -980,17 +981,17 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>mentor_comment</t>
+          <t>learning_note</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>导师点评表</t>
+          <t>学习笔记表</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>师承关系中的权威内容。is_ai_generated 字段确保 AI 生成内容绝不被误认为真实导师点评，界面须视觉区分。</t>
+          <t>以 note_type 区分跟诊日志与学习心得，避免为相似结构建多张表。</t>
         </is>
       </c>
     </row>
@@ -1005,17 +1006,17 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>note_record_link</t>
+          <t>mentor_comment</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>笔记与病案关联表</t>
+          <t>导师点评表</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>学习心得与病案的双向引用，支持“从心得跳病案”与反向追溯。</t>
+          <t>师承关系中的权威内容。is_ai_generated 字段确保 AI 生成内容绝不被误认为真实导师点评，界面须视觉区分。</t>
         </is>
       </c>
     </row>
@@ -1025,22 +1026,22 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>六、来源与溯源</t>
+          <t>五、跟师学习</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>source_document</t>
+          <t>note_record_link</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>来源单据表</t>
+          <t>笔记与病案关联表</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>真实样本显示同一病程的数据可能来自手写教学表单、HIS 打印件或 HIS 界面截图，来源不同则解析策略与可信度不同。</t>
+          <t>学习心得与病案的双向引用，支持“从心得跳病案”与反向追溯。</t>
         </is>
       </c>
     </row>
@@ -1055,17 +1056,17 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>attachment</t>
+          <t>source_document</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>附件表</t>
+          <t>来源单据表</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>文件本体存于 data/attachments/，库中仅存路径与哈希。sha256 用于去重与完整性校验。</t>
+          <t>真实样本显示同一病程的数据可能来自手写教学表单、HIS 打印件或 HIS 界面截图，来源不同则解析策略与可信度不同。</t>
         </is>
       </c>
     </row>
@@ -1080,17 +1081,17 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>ocr_job</t>
+          <t>attachment</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>OCR作业表</t>
+          <t>附件表</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>一次识别的完整留痕：双通道结果、提示词版本、成本与耗时。提示词固定前缀须字节级稳定以命中 DeepSeek 上下文缓存。</t>
+          <t>文件本体存于 data/attachments/，库中仅存路径与哈希。sha256 用于去重与完整性校验。</t>
         </is>
       </c>
     </row>
@@ -1105,17 +1106,17 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>ocr_field_confidence</t>
+          <t>ocr_job</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>OCR字段置信度表</t>
+          <t>OCR作业表</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>驱动校对界面高亮，同时是 OCR 评测的数据来源。真实样本显示印刷体置信度0.5~1.0、手写体约0.3，可据此路由。</t>
+          <t>一次识别的完整留痕：双通道结果、提示词版本、成本与耗时。提示词固定前缀须字节级稳定以命中 DeepSeek 上下文缓存。</t>
         </is>
       </c>
     </row>
@@ -1125,22 +1126,22 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>七、系统</t>
+          <t>六、来源与溯源</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>audit_log</t>
+          <t>ocr_field_confidence</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>审计日志表</t>
+          <t>OCR字段置信度表</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>字段级修改留痕。学习记录的可信性依赖不可抵赖的修改历史。</t>
+          <t>驱动校对界面高亮，同时是 OCR 评测的数据来源。真实样本显示印刷体置信度0.5~1.0、手写体约0.3，可据此路由。</t>
         </is>
       </c>
     </row>
@@ -1155,15 +1156,40 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
+          <t>audit_log</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>审计日志表</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>字段级修改留痕。学习记录的可信性依赖不可抵赖的修改历史。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>七、系统</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
           <t>app_setting</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>应用设置表</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="E29" s="4" t="inlineStr">
         <is>
           <t>仅存非敏感偏好。API Key 等敏感项存于 .env，不入库、不入 Git。</t>
         </is>
@@ -1489,6 +1515,365 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>西药明细表（western_medicine_item）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>结构化存储西药处方，一行一味：药名、剂量、给药途径、给药频次与天数。可由 OCR 从医嘱单中识别入库。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>字段名称</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>中文释义</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>数据类型（SQLite）</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>键描述</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>数据说明与数据约束</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>wm_id</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>西药明细编号</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>PRIMARY KEY AUTOINCREMENT</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>计算机生成：从1开始，以1为步长增序编号</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>record_id</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>病历编号</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>FOREIGN KEY</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>必填，关联 info_record</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>patient_id</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>患者编号</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>FOREIGN KEY</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>计算机生成，与患者基本信息同步记录</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>drug_name</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>药名</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>必填，如“甲钴胺”“加巴喷丁”</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>dose</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>剂量</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>选填，如“0.5mg”“1片”“10ml”</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>给药途径</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>选填，如“口服”“静脉滴注”，建议取值见 dict_term（类型=给药途径）</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>frequency</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>给药频次</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>选填，如“tid”“bid”“每日三次”，建议取值见 dict_term（类型=给药频次）</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>天数</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>选填，如“7天”“14”</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>needs_review</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>是否待校对</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>BOOLEAN</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>0为正常，1为需人工复核</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>confidence</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>识别置信度</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>REAL</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 1</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>选填，人工录入为1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>创建时间</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr"/>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录创建时间</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1977,7 +2362,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2228,7 +2613,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2587,7 +2972,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2973,7 +3358,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3282,7 +3667,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3533,7 +3918,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3915,7 +4300,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4206,230 +4591,6 @@
       </c>
       <c r="D12" s="4" t="inlineStr"/>
       <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录创建时间</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="62" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>笔记与病案关联表（note_record_link）</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>学习心得与病案的双向引用，支持“从心得跳病案”与反向追溯。</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>字段名称</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>中文释义</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>数据类型（SQLite）</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>键描述</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>数据说明与数据约束</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>link_id</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>关联编号</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>INTEGER</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>PRIMARY KEY AUTOINCREMENT</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>计算机生成：从1开始，以1为步长增序编号</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>note_id</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>笔记编号</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>FOREIGN KEY NOT NULL</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>必填，关联 learning_note</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>record_id</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>病历编号</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>INTEGER</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>FOREIGN KEY NOT NULL</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>必填，关联 info_record</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>relation</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>关联类型</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>UNSIGNED TINYINT</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT 0</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>0为引证，1为讨论，2为对比；详见附表A10</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>notes</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>说明</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>DEFAULT ''</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>选填，默认为空字符串</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>创建时间</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>TIMESTAMP</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr"/>
-      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录创建时间</t>
         </is>
@@ -4940,6 +5101,230 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>笔记与病案关联表（note_record_link）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>学习心得与病案的双向引用，支持“从心得跳病案”与反向追溯。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>字段名称</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>中文释义</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>数据类型（SQLite）</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>键描述</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>数据说明与数据约束</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>link_id</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>关联编号</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>PRIMARY KEY AUTOINCREMENT</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>计算机生成：从1开始，以1为步长增序编号</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>note_id</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>笔记编号</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>FOREIGN KEY NOT NULL</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>必填，关联 learning_note</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>record_id</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>病历编号</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>FOREIGN KEY NOT NULL</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>必填，关联 info_record</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>relation</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>关联类型</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>UNSIGNED TINYINT</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>0为引证，1为讨论，2为对比；详见附表A10</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>说明</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>选填，默认为空字符串</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>创建时间</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>计算机以“%Y-%m-%d %H:%M:%S”形式自动存储记录创建时间</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5239,7 +5624,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5706,7 +6091,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6329,7 +6714,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6661,7 +7046,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6970,7 +7355,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7113,7 +7498,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7232,7 +7617,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>1=舌质；2=舌苔；3=脉象；4=面色；5=炮制；6=煎服法；7=用法；8=中医病名；9=治法；10=剂型；11=特殊煎煮法</t>
+          <t>1=舌质；2=舌苔；3=脉象；4=面色；5=炮制；6=煎服法；7=用法；8=中医病名；9=治法；10=剂型；11=特殊煎煮法；12=给药途径；13=给药频次</t>
         </is>
       </c>
     </row>

</xml_diff>